<commit_message>
Use black bold totals instead of red on Yellowstone monthly budget
Co-authored-by: crios82-max <crios82-max@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/presupuesto-yellowstone-gerencia-mensual.xlsx
+++ b/docs/presupuesto-yellowstone-gerencia-mensual.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,19 +76,25 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00111111"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00111A2D"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00C41E3A"/>
+      <color rgb="00111111"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00C41E3A"/>
+      <color rgb="00111111"/>
       <sz val="14"/>
     </font>
     <font>
@@ -104,7 +110,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -123,7 +129,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF5F5"/>
+        <fgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -134,11 +140,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -187,13 +188,13 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -201,15 +202,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>

</xml_diff>

<commit_message>
Align monthly Yellowstone budget to organigram concepts
Replace prior personal/staff/gerencia expense lines with organigram
structure items (general management, regional units, capacity and
account goal) while keeping the USD 64,248 monthly total.

Co-authored-by: crios82-max <crios82-max@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/presupuesto-yellowstone-gerencia-mensual.xlsx
+++ b/docs/presupuesto-yellowstone-gerencia-mensual.xlsx
@@ -65,13 +65,13 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00151A22"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00151A22"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -99,15 +99,14 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="005F6874"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00111A2D"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="0094A3B8"/>
-      <sz val="8"/>
     </font>
   </fonts>
   <fills count="7">
@@ -186,7 +185,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -201,16 +200,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -576,12 +577,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D26"/>
+  <dimension ref="B2:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -595,14 +596,14 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Operación mensual de cuentas orgánicas + estructura</t>
+          <t>Estructura actual · operación mensual</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Red Humana, Espartanos, Laboratorio Bots, Staff y Equipo de Gerencia</t>
+          <t>Sin líneas de personal/staff ni equipo de gerencia · conceptos de organigrama</t>
         </is>
       </c>
     </row>
@@ -636,160 +637,150 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="26" customHeight="1">
+    <row r="9" ht="28" customHeight="1">
       <c r="B9" s="8" t="n">
-        <v>9000</v>
+        <v>1</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>RED HUMANA (operación mensual)</t>
+          <t>GERENCIA GENERAL</t>
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>29850</v>
-      </c>
-    </row>
-    <row r="10" ht="26" customHeight="1">
+        <v>8450</v>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
       <c r="B10" s="8" t="n">
-        <v>3000</v>
+        <v>24</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>BOTS ORIGINALES (mantenimiento mensual)</t>
+          <t>GERENCIAS REGIONALES (4 gerentes x 6 regiones)</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>15450</v>
-      </c>
-    </row>
-    <row r="11" ht="26" customHeight="1">
+        <v>18600</v>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
       <c r="B11" s="8" t="n">
-        <v>500</v>
+        <v>1512</v>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>ESPARTANOS (operación elite mensual)</t>
+          <t>ESTRUCTURA OPERATIVA (24 gerencias x 63 personas)</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>10200</v>
-      </c>
-    </row>
-    <row r="12" ht="26" customHeight="1">
+        <v>22848</v>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
       <c r="B12" s="8" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>LABORATORIO BOTS (soporte mensual)</t>
+          <t>CUENTAS POR PERSONA (capacidad operativa)</t>
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>4248</v>
-      </c>
-    </row>
-    <row r="13" ht="26" customHeight="1">
+        <v>9200</v>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
       <c r="B13" s="8" t="n">
-        <v>12</v>
+        <v>15120</v>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>STAFF (operación mensual)</t>
+          <t>META DE CUENTAS (1.512 personas x 10 cuentas)</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>3148</v>
-      </c>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="B14" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>EQUIPO GERENCIA (dirección mensual)</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="n">
-        <v>1352</v>
-      </c>
-    </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="B16" s="11" t="inlineStr">
+        <v>5150</v>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>TOTAL GERENCIA MENSUAL</t>
         </is>
       </c>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="12" t="n">
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="12" t="n">
         <v>64248</v>
       </c>
     </row>
+    <row r="17">
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>RESUMEN</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="14" t="n"/>
+    </row>
     <row r="18">
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>RESUMEN</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>Inversión mensual</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="16" t="n">
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="16" t="n">
         <v>64248</v>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="17" t="inlineStr">
+    <row r="20" ht="28" customHeight="1">
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Referencia estructura: estatus actual 9.634 cuentas · 63,72% avance · 5.486 por alcanzar (sin costo adicional en este presupuesto).</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="n"/>
+      <c r="D20" s="18" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>• Presupuesto de gerencia mensual Yellowstone (operación continua).
+    <row r="23">
+      <c r="B23" s="20" t="inlineStr">
+        <is>
+          <t>• Conceptos alineados al organigrama. Se eliminaron gastos de personal/staff y equipo de gerencia.
 • Validez del presupuesto: 15 días. Montos en dólares estadounidenses (USD).
 • Total gerencia mensual: USD 64,248.</t>
         </is>
       </c>
-      <c r="C22" s="19" t="n"/>
-      <c r="D22" s="19" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="19" t="n"/>
-      <c r="C23" s="19" t="n"/>
-      <c r="D23" s="19" t="n"/>
+      <c r="C23" s="18" t="n"/>
+      <c r="D23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="19" t="n"/>
-      <c r="C24" s="19" t="n"/>
-      <c r="D24" s="19" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="20" t="inlineStr">
-        <is>
-          <t>YELLOWSTONE · Gerencia mensual · 1 hoja</t>
-        </is>
-      </c>
+      <c r="B24" s="18" t="n"/>
+      <c r="C24" s="18" t="n"/>
+      <c r="D24" s="18" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="18" t="n"/>
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="18" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B22:D24"/>
-    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B15:C15"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B23:D25"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:C18"/>
     <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B20:D20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refine organigram monthly budget layout and concept labels
Co-authored-by: crios82-max <crios82-max@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/presupuesto-yellowstone-gerencia-mensual.xlsx
+++ b/docs/presupuesto-yellowstone-gerencia-mensual.xlsx
@@ -185,7 +185,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -204,9 +204,7 @@
     <xf numFmtId="164" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -582,7 +580,7 @@
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -603,7 +601,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Sin líneas de personal/staff ni equipo de gerencia · conceptos de organigrama</t>
+          <t>Conceptos del organigrama (sin líneas de personal ni gerencia operativa)</t>
         </is>
       </c>
     </row>
@@ -637,7 +635,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="26" customHeight="1">
       <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
@@ -650,52 +648,52 @@
         <v>8450</v>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="26" customHeight="1">
       <c r="B10" s="8" t="n">
         <v>24</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>GERENCIAS REGIONALES (4 gerentes x 6 regiones)</t>
+          <t>GERENCIAS REGIONALES (4 x 6 regiones)</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
         <v>18600</v>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="26" customHeight="1">
       <c r="B11" s="8" t="n">
         <v>1512</v>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>ESTRUCTURA OPERATIVA (24 gerencias x 63 personas)</t>
+          <t>ESTRUCTURA OPERATIVA (24 x 63)</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
         <v>22848</v>
       </c>
     </row>
-    <row r="12" ht="28" customHeight="1">
+    <row r="12" ht="26" customHeight="1">
       <c r="B12" s="8" t="n">
         <v>10</v>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>CUENTAS POR PERSONA (capacidad operativa)</t>
+          <t>CUENTAS POR PERSONA (capacidad)</t>
         </is>
       </c>
       <c r="D12" s="10" t="n">
         <v>9200</v>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="26" customHeight="1">
       <c r="B13" s="8" t="n">
         <v>15120</v>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>META DE CUENTAS (1.512 personas x 10 cuentas)</t>
+          <t>META DE CUENTAS (1.512 x 10)</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
@@ -733,10 +731,10 @@
         <v>64248</v>
       </c>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20">
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Referencia estructura: estatus actual 9.634 cuentas · 63,72% avance · 5.486 por alcanzar (sin costo adicional en este presupuesto).</t>
+          <t>Referencia: estatus 9.634 cuentas · 63,72% avance · 5.486 por alcanzar (sin costo extra).</t>
         </is>
       </c>
       <c r="C20" s="18" t="n"/>
@@ -752,7 +750,7 @@
     <row r="23">
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>• Conceptos alineados al organigrama. Se eliminaron gastos de personal/staff y equipo de gerencia.
+          <t>• Conceptos alineados al organigrama de estructura actual.
 • Validez del presupuesto: 15 días. Montos en dólares estadounidenses (USD).
 • Total gerencia mensual: USD 64,248.</t>
         </is>

</xml_diff>

<commit_message>
Drop account-capacity lines and redistribute monthly total
Remove cuentas por persona and meta de cuentas from the Yellowstone
monthly budget and allocate their amounts across the remaining
organigram items, keeping USD 64,248.

Co-authored-by: crios82-max <crios82-max@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/presupuesto-yellowstone-gerencia-mensual.xlsx
+++ b/docs/presupuesto-yellowstone-gerencia-mensual.xlsx
@@ -575,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D25"/>
+  <dimension ref="B2:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -601,7 +601,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Conceptos del organigrama (sin líneas de personal ni gerencia operativa)</t>
+          <t>Conceptos del organigrama (sin cuentas por persona ni meta de cuentas)</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>8450</v>
+        <v>11450</v>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>18600</v>
+        <v>23600</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
@@ -671,114 +671,88 @@
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>22848</v>
-      </c>
-    </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="B12" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>CUENTAS POR PERSONA (capacidad)</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="n">
-        <v>9200</v>
-      </c>
-    </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="B13" s="8" t="n">
-        <v>15120</v>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>META DE CUENTAS (1.512 x 10)</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="n">
-        <v>5150</v>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="B15" s="11" t="inlineStr">
+        <v>29198</v>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>TOTAL GERENCIA MENSUAL</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="12" t="n">
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="12" t="n">
         <v>64248</v>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="13" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>RESUMEN</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="14" t="n"/>
+      <c r="C15" s="14" t="n"/>
+      <c r="D15" s="14" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Inversión mensual</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="16" t="n">
+        <v>64248</v>
+      </c>
     </row>
     <row r="18">
-      <c r="B18" s="15" t="inlineStr">
-        <is>
-          <t>Inversión mensual</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="16" t="n">
-        <v>64248</v>
-      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>Referencia: estatus 9.634 cuentas · 63,72% avance · 5.486 por alcanzar (sin costo extra).</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="n"/>
+      <c r="D18" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>Referencia: estatus 9.634 cuentas · 63,72% avance · 5.486 por alcanzar (sin costo extra).</t>
-        </is>
-      </c>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="18" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="19" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="20" t="inlineStr">
-        <is>
-          <t>• Conceptos alineados al organigrama de estructura actual.
+    <row r="21">
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>• Sin líneas de cuentas por persona ni meta de cuentas; monto redistribuido.
 • Validez del presupuesto: 15 días. Montos en dólares estadounidenses (USD).
 • Total gerencia mensual: USD 64,248.</t>
         </is>
       </c>
+      <c r="C21" s="18" t="n"/>
+      <c r="D21" s="18" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="18" t="n"/>
+      <c r="C22" s="18" t="n"/>
+      <c r="D22" s="18" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="18" t="n"/>
       <c r="C23" s="18" t="n"/>
       <c r="D23" s="18" t="n"/>
     </row>
-    <row r="24">
-      <c r="B24" s="18" t="n"/>
-      <c r="C24" s="18" t="n"/>
-      <c r="D24" s="18" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="18" t="n"/>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="18" t="n"/>
-    </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B13:C13"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B23:D25"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B21:D23"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B20:D20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>